<commit_message>
updates from MMCF 2025 project: DCC, FIC, techs, carbon taxes, NZ fuel prices (from CER), OBPS, source files
</commit_message>
<xml_diff>
--- a/csv/model/DCC/formula_DCC_ON.xlsx
+++ b/csv/model/DCC/formula_DCC_ON.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CIMS\dev\cims-models\csv\model\DCC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CIMS\test\cims-models\csv\model\DCC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A177E115-57ED-4812-9B54-6DAF2F0B1D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{73033F45-3305-4047-BBC2-0CD78EDECD92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72F828C2-0B44-41B3-B3F5-7C3BEA2525F4}"/>
+    <workbookView xWindow="32505" yWindow="2025" windowWidth="38700" windowHeight="15285" xr2:uid="{82E3A5A0-5571-491E-ABF7-3A3E3478C04D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -985,16 +985,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC09DFFA-C805-42D8-8B02-D20094685CB1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB8D82AB-79E8-47A7-BA54-EE3C90D3BE26}">
   <dimension ref="A1:X488"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1127,7 +1127,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1186,7 +1186,7 @@
         <v>10.6</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -1422,7 +1422,7 @@
         <v>3.62</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>17.009699999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>6840</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>25000</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -1658,7 +1658,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>48</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>48</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -1838,50 +1838,50 @@
         <v>54</v>
       </c>
       <c r="M16">
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="N16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="O16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="P16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="Q16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="R16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="S16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="T16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="U16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="V16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="W16">
         <f t="shared" ca="1" si="0"/>
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>48</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -1976,50 +1976,50 @@
         <v>54</v>
       </c>
       <c r="M18">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="N18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="O18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="P18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="Q18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="R18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="S18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="T18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="U18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="V18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="W18">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>48</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>48</v>
       </c>
@@ -2114,7 +2114,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -2183,7 +2183,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>48</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>48</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>48</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>48</v>
       </c>
@@ -2416,7 +2416,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>48</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>48</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>48</v>
       </c>
@@ -2649,7 +2649,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>48</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>48</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>48</v>
       </c>
@@ -2856,7 +2856,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>48</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>48</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>48</v>
       </c>
@@ -3020,7 +3020,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>48</v>
       </c>
@@ -3046,50 +3046,50 @@
         <v>54</v>
       </c>
       <c r="M36">
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="N36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="O36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="P36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="Q36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="R36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="S36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="T36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="U36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="V36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="W36">
         <f t="shared" ca="1" si="4"/>
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>48</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>48</v>
       </c>
@@ -3184,50 +3184,50 @@
         <v>54</v>
       </c>
       <c r="M38">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="N38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="O38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="P38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="Q38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="R38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="S38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="T38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="U38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="V38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="W38">
         <f t="shared" ca="1" si="4"/>
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>48</v>
       </c>
@@ -3253,7 +3253,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>48</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>48</v>
       </c>
@@ -3391,7 +3391,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>48</v>
       </c>
@@ -3460,7 +3460,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -3529,7 +3529,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>48</v>
       </c>
@@ -3624,7 +3624,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>48</v>
       </c>
@@ -3693,7 +3693,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>48</v>
       </c>
@@ -3762,7 +3762,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>48</v>
       </c>
@@ -3831,7 +3831,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>67</v>
       </c>
@@ -3857,7 +3857,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>67</v>
       </c>
@@ -3926,7 +3926,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>67</v>
       </c>
@@ -3952,50 +3952,50 @@
         <v>54</v>
       </c>
       <c r="M51">
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="N51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="O51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="P51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="Q51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="R51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="S51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="T51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="U51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="V51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="W51">
         <f t="shared" ca="1" si="7"/>
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>67</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>67</v>
       </c>
@@ -4090,50 +4090,50 @@
         <v>54</v>
       </c>
       <c r="M53">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="N53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="O53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="P53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="Q53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="R53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="S53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="T53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="U53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="V53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="W53">
         <f t="shared" ca="1" si="7"/>
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>67</v>
       </c>
@@ -4159,7 +4159,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>67</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>67</v>
       </c>
@@ -4297,7 +4297,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>67</v>
       </c>
@@ -4366,7 +4366,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>67</v>
       </c>
@@ -4435,7 +4435,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>67</v>
       </c>
@@ -4461,7 +4461,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>67</v>
       </c>
@@ -4530,7 +4530,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -4599,7 +4599,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>67</v>
       </c>
@@ -4668,7 +4668,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>67</v>
       </c>
@@ -4737,7 +4737,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>69</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>69</v>
       </c>
@@ -4832,7 +4832,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>69</v>
       </c>
@@ -4901,7 +4901,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>69</v>
       </c>
@@ -4970,7 +4970,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>69</v>
       </c>
@@ -5039,7 +5039,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>71</v>
       </c>
@@ -5065,7 +5065,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>71</v>
       </c>
@@ -5134,7 +5134,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>71</v>
       </c>
@@ -5203,7 +5203,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -5272,7 +5272,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>71</v>
       </c>
@@ -5341,7 +5341,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>73</v>
       </c>
@@ -5367,7 +5367,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="75" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>73</v>
       </c>
@@ -5436,7 +5436,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="76" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>73</v>
       </c>
@@ -5505,7 +5505,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="77" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>73</v>
       </c>
@@ -5574,7 +5574,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="78" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>73</v>
       </c>
@@ -5643,7 +5643,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="79" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>75</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="80" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>75</v>
       </c>
@@ -5738,7 +5738,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>75</v>
       </c>
@@ -5807,7 +5807,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>75</v>
       </c>
@@ -5877,7 +5877,7 @@
         <v>2861100</v>
       </c>
     </row>
-    <row r="83" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>75</v>
       </c>
@@ -5946,7 +5946,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="84" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>79</v>
       </c>
@@ -5972,7 +5972,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="85" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>79</v>
       </c>
@@ -6041,7 +6041,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="86" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>79</v>
       </c>
@@ -6110,7 +6110,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="87" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>79</v>
       </c>
@@ -6180,7 +6180,7 @@
         <v>2861100</v>
       </c>
     </row>
-    <row r="88" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>79</v>
       </c>
@@ -6249,7 +6249,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="89" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>81</v>
       </c>
@@ -6275,7 +6275,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="90" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>81</v>
       </c>
@@ -6344,7 +6344,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="91" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>81</v>
       </c>
@@ -6413,7 +6413,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="92" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>81</v>
       </c>
@@ -6483,7 +6483,7 @@
         <v>2861100</v>
       </c>
     </row>
-    <row r="93" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>81</v>
       </c>
@@ -6552,7 +6552,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="94" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>83</v>
       </c>
@@ -6578,7 +6578,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="95" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>83</v>
       </c>
@@ -6647,7 +6647,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="96" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>83</v>
       </c>
@@ -6716,7 +6716,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="97" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>83</v>
       </c>
@@ -6786,7 +6786,7 @@
         <v>7668000</v>
       </c>
     </row>
-    <row r="98" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>83</v>
       </c>
@@ -6855,7 +6855,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="99" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>88</v>
       </c>
@@ -6881,7 +6881,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="100" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>88</v>
       </c>
@@ -6950,7 +6950,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="101" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>88</v>
       </c>
@@ -7019,7 +7019,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="102" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>88</v>
       </c>
@@ -7092,7 +7092,7 @@
         <v>50000000</v>
       </c>
     </row>
-    <row r="103" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>88</v>
       </c>
@@ -7161,7 +7161,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="104" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>88</v>
       </c>
@@ -7187,7 +7187,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="105" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>88</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="106" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>88</v>
       </c>
@@ -7325,7 +7325,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="107" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>88</v>
       </c>
@@ -7398,7 +7398,7 @@
         <v>125000000</v>
       </c>
     </row>
-    <row r="108" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>88</v>
       </c>
@@ -7467,7 +7467,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="109" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>88</v>
       </c>
@@ -7493,7 +7493,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="110" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>88</v>
       </c>
@@ -7562,7 +7562,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="111" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>88</v>
       </c>
@@ -7631,7 +7631,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="112" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>88</v>
       </c>
@@ -7704,7 +7704,7 @@
         <v>125000000</v>
       </c>
     </row>
-    <row r="113" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>88</v>
       </c>
@@ -7773,7 +7773,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="114" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>88</v>
       </c>
@@ -7799,7 +7799,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="115" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>88</v>
       </c>
@@ -7868,7 +7868,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="116" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>88</v>
       </c>
@@ -7937,7 +7937,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="117" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>88</v>
       </c>
@@ -8010,7 +8010,7 @@
         <v>50000000</v>
       </c>
     </row>
-    <row r="118" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>88</v>
       </c>
@@ -8079,7 +8079,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="119" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>88</v>
       </c>
@@ -8105,7 +8105,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="120" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>88</v>
       </c>
@@ -8174,7 +8174,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="121" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>88</v>
       </c>
@@ -8243,7 +8243,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="122" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>88</v>
       </c>
@@ -8316,7 +8316,7 @@
         <v>50000000</v>
       </c>
     </row>
-    <row r="123" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>88</v>
       </c>
@@ -8385,7 +8385,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="124" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>88</v>
       </c>
@@ -8411,7 +8411,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="125" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>88</v>
       </c>
@@ -8480,7 +8480,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="126" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>88</v>
       </c>
@@ -8549,7 +8549,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="127" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>88</v>
       </c>
@@ -8622,7 +8622,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="128" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>88</v>
       </c>
@@ -8691,7 +8691,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="129" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>88</v>
       </c>
@@ -8717,7 +8717,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="130" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>88</v>
       </c>
@@ -8786,7 +8786,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="131" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>88</v>
       </c>
@@ -8855,7 +8855,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="132" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>88</v>
       </c>
@@ -8928,7 +8928,7 @@
         <v>125000000</v>
       </c>
     </row>
-    <row r="133" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>88</v>
       </c>
@@ -8997,7 +8997,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="134" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>88</v>
       </c>
@@ -9023,7 +9023,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="135" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>88</v>
       </c>
@@ -9092,7 +9092,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="136" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>88</v>
       </c>
@@ -9161,7 +9161,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="137" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>88</v>
       </c>
@@ -9234,7 +9234,7 @@
         <v>50000000</v>
       </c>
     </row>
-    <row r="138" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>88</v>
       </c>
@@ -9303,7 +9303,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="139" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>88</v>
       </c>
@@ -9329,7 +9329,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="140" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>88</v>
       </c>
@@ -9398,7 +9398,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="141" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>88</v>
       </c>
@@ -9467,7 +9467,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="142" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>88</v>
       </c>
@@ -9540,7 +9540,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="143" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>88</v>
       </c>
@@ -9609,7 +9609,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="144" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>105</v>
       </c>
@@ -9635,7 +9635,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="145" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>105</v>
       </c>
@@ -9704,7 +9704,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="146" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>105</v>
       </c>
@@ -9773,7 +9773,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="147" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>105</v>
       </c>
@@ -9846,7 +9846,7 @@
         <v>200000000</v>
       </c>
     </row>
-    <row r="148" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>105</v>
       </c>
@@ -9915,7 +9915,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="149" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>109</v>
       </c>
@@ -9941,7 +9941,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="150" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>109</v>
       </c>
@@ -10010,7 +10010,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="151" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>109</v>
       </c>
@@ -10079,7 +10079,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="152" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>109</v>
       </c>
@@ -10149,7 +10149,7 @@
         <v>2861100</v>
       </c>
     </row>
-    <row r="153" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>109</v>
       </c>
@@ -10218,7 +10218,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="154" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>110</v>
       </c>
@@ -10244,7 +10244,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="155" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>110</v>
       </c>
@@ -10313,7 +10313,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="156" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>110</v>
       </c>
@@ -10382,7 +10382,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="157" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>110</v>
       </c>
@@ -10452,7 +10452,7 @@
         <v>2861100</v>
       </c>
     </row>
-    <row r="158" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>110</v>
       </c>
@@ -10521,7 +10521,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="159" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>112</v>
       </c>
@@ -10547,7 +10547,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="160" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>112</v>
       </c>
@@ -10616,7 +10616,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="161" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>112</v>
       </c>
@@ -10685,7 +10685,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="162" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>112</v>
       </c>
@@ -10754,7 +10754,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="163" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>112</v>
       </c>
@@ -10823,7 +10823,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="164" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>112</v>
       </c>
@@ -10849,7 +10849,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="165" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>112</v>
       </c>
@@ -10918,7 +10918,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="166" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>112</v>
       </c>
@@ -10987,7 +10987,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="167" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>112</v>
       </c>
@@ -11056,7 +11056,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="168" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>112</v>
       </c>
@@ -11125,7 +11125,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="169" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>120</v>
       </c>
@@ -11151,7 +11151,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="170" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>120</v>
       </c>
@@ -11220,7 +11220,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="171" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>120</v>
       </c>
@@ -11289,7 +11289,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="172" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>120</v>
       </c>
@@ -11358,7 +11358,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="173" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>120</v>
       </c>
@@ -11427,7 +11427,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="174" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>120</v>
       </c>
@@ -11453,7 +11453,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="175" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>120</v>
       </c>
@@ -11522,7 +11522,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="176" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>120</v>
       </c>
@@ -11591,7 +11591,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="177" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>120</v>
       </c>
@@ -11660,7 +11660,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="178" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>120</v>
       </c>
@@ -11729,7 +11729,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="179" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>122</v>
       </c>
@@ -11755,7 +11755,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="180" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>122</v>
       </c>
@@ -11824,7 +11824,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="181" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>122</v>
       </c>
@@ -11893,7 +11893,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="182" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>122</v>
       </c>
@@ -11963,7 +11963,7 @@
         <v>2861100</v>
       </c>
     </row>
-    <row r="183" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>122</v>
       </c>
@@ -12032,7 +12032,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="184" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>123</v>
       </c>
@@ -12058,7 +12058,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="185" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>123</v>
       </c>
@@ -12127,7 +12127,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="186" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>123</v>
       </c>
@@ -12196,7 +12196,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="187" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>123</v>
       </c>
@@ -12265,7 +12265,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="188" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>123</v>
       </c>
@@ -12334,7 +12334,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="189" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>128</v>
       </c>
@@ -12360,7 +12360,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="190" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>128</v>
       </c>
@@ -12429,7 +12429,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="191" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>128</v>
       </c>
@@ -12498,7 +12498,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="192" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>128</v>
       </c>
@@ -12568,7 +12568,7 @@
         <v>2861100</v>
       </c>
     </row>
-    <row r="193" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>128</v>
       </c>
@@ -12637,7 +12637,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="194" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>129</v>
       </c>
@@ -12663,7 +12663,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="195" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>129</v>
       </c>
@@ -12689,7 +12689,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="196" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>135</v>
       </c>
@@ -12715,7 +12715,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="197" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>135</v>
       </c>
@@ -12741,7 +12741,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="198" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>136</v>
       </c>
@@ -12767,7 +12767,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="199" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>136</v>
       </c>
@@ -12793,7 +12793,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="200" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>137</v>
       </c>
@@ -12819,7 +12819,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="201" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>137</v>
       </c>
@@ -12845,7 +12845,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="202" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>137</v>
       </c>
@@ -12871,7 +12871,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="203" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>139</v>
       </c>
@@ -12897,7 +12897,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="204" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>139</v>
       </c>
@@ -12923,7 +12923,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="205" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>139</v>
       </c>
@@ -12949,7 +12949,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="206" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>140</v>
       </c>
@@ -12975,7 +12975,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="207" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>140</v>
       </c>
@@ -13001,7 +13001,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="208" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>140</v>
       </c>
@@ -13027,7 +13027,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="209" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>141</v>
       </c>
@@ -13053,7 +13053,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="210" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>141</v>
       </c>
@@ -13079,7 +13079,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="211" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>142</v>
       </c>
@@ -13105,7 +13105,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="212" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>142</v>
       </c>
@@ -13131,7 +13131,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="213" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>143</v>
       </c>
@@ -13157,7 +13157,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="214" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>143</v>
       </c>
@@ -13183,7 +13183,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="215" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>144</v>
       </c>
@@ -13209,7 +13209,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="216" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>144</v>
       </c>
@@ -13235,7 +13235,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="217" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>145</v>
       </c>
@@ -13261,7 +13261,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="218" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>145</v>
       </c>
@@ -13287,7 +13287,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="219" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>146</v>
       </c>
@@ -13313,7 +13313,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="220" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>146</v>
       </c>
@@ -13339,7 +13339,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="221" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>129</v>
       </c>
@@ -13395,7 +13395,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="222" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>129</v>
       </c>
@@ -13451,7 +13451,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="223" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>135</v>
       </c>
@@ -13507,7 +13507,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="224" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>135</v>
       </c>
@@ -13563,7 +13563,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="225" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>136</v>
       </c>
@@ -13619,7 +13619,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="226" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>136</v>
       </c>
@@ -13675,7 +13675,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="227" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>137</v>
       </c>
@@ -13731,7 +13731,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="228" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>137</v>
       </c>
@@ -13787,7 +13787,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="229" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>137</v>
       </c>
@@ -13843,7 +13843,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="230" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>139</v>
       </c>
@@ -13899,7 +13899,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="231" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>139</v>
       </c>
@@ -13955,7 +13955,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="232" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>139</v>
       </c>
@@ -14011,7 +14011,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="233" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>140</v>
       </c>
@@ -14067,7 +14067,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="234" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>140</v>
       </c>
@@ -14123,7 +14123,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="235" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>140</v>
       </c>
@@ -14179,7 +14179,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="236" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>141</v>
       </c>
@@ -14235,7 +14235,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="237" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>141</v>
       </c>
@@ -14291,7 +14291,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="238" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>142</v>
       </c>
@@ -14347,7 +14347,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="239" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>142</v>
       </c>
@@ -14403,7 +14403,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="240" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>143</v>
       </c>
@@ -14459,7 +14459,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="241" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>143</v>
       </c>
@@ -14515,7 +14515,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="242" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>144</v>
       </c>
@@ -14571,7 +14571,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="243" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>144</v>
       </c>
@@ -14627,7 +14627,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="244" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>145</v>
       </c>
@@ -14683,7 +14683,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="245" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>145</v>
       </c>
@@ -14739,7 +14739,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="246" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>146</v>
       </c>
@@ -14795,7 +14795,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="247" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>146</v>
       </c>
@@ -14851,7 +14851,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="248" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>129</v>
       </c>
@@ -14907,7 +14907,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="249" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>129</v>
       </c>
@@ -14963,7 +14963,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="250" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>135</v>
       </c>
@@ -15019,7 +15019,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="251" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>135</v>
       </c>
@@ -15075,7 +15075,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="252" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>136</v>
       </c>
@@ -15131,7 +15131,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="253" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>136</v>
       </c>
@@ -15187,7 +15187,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="254" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>137</v>
       </c>
@@ -15243,7 +15243,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="255" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>137</v>
       </c>
@@ -15299,7 +15299,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="256" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>137</v>
       </c>
@@ -15355,7 +15355,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="257" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>139</v>
       </c>
@@ -15411,7 +15411,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="258" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>139</v>
       </c>
@@ -15467,7 +15467,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="259" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>139</v>
       </c>
@@ -15523,7 +15523,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="260" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>140</v>
       </c>
@@ -15579,7 +15579,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="261" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>140</v>
       </c>
@@ -15635,7 +15635,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="262" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>140</v>
       </c>
@@ -15691,7 +15691,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="263" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>141</v>
       </c>
@@ -15747,7 +15747,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="264" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>141</v>
       </c>
@@ -15803,7 +15803,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="265" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>142</v>
       </c>
@@ -15859,7 +15859,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="266" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>142</v>
       </c>
@@ -15915,7 +15915,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="267" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>143</v>
       </c>
@@ -15971,7 +15971,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="268" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>143</v>
       </c>
@@ -16027,7 +16027,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="269" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>144</v>
       </c>
@@ -16083,7 +16083,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="270" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>144</v>
       </c>
@@ -16139,7 +16139,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="271" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>145</v>
       </c>
@@ -16195,7 +16195,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="272" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>145</v>
       </c>
@@ -16251,7 +16251,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="273" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>146</v>
       </c>
@@ -16307,7 +16307,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="274" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>146</v>
       </c>
@@ -16363,7 +16363,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="275" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>129</v>
       </c>
@@ -16419,7 +16419,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="276" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>129</v>
       </c>
@@ -16475,7 +16475,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="277" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>135</v>
       </c>
@@ -16531,7 +16531,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="278" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>135</v>
       </c>
@@ -16587,7 +16587,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="279" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>136</v>
       </c>
@@ -16643,7 +16643,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="280" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>136</v>
       </c>
@@ -16699,7 +16699,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="281" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>137</v>
       </c>
@@ -16755,7 +16755,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="282" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>137</v>
       </c>
@@ -16811,7 +16811,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="283" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>137</v>
       </c>
@@ -16867,7 +16867,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="284" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>139</v>
       </c>
@@ -16923,7 +16923,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="285" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>139</v>
       </c>
@@ -16979,7 +16979,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="286" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>139</v>
       </c>
@@ -17035,7 +17035,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="287" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>140</v>
       </c>
@@ -17091,7 +17091,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="288" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>140</v>
       </c>
@@ -17147,7 +17147,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="289" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>140</v>
       </c>
@@ -17203,7 +17203,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="290" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>141</v>
       </c>
@@ -17259,7 +17259,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="291" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>141</v>
       </c>
@@ -17315,7 +17315,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="292" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>142</v>
       </c>
@@ -17371,7 +17371,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="293" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>142</v>
       </c>
@@ -17427,7 +17427,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="294" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>143</v>
       </c>
@@ -17483,7 +17483,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="295" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>143</v>
       </c>
@@ -17539,7 +17539,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="296" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>144</v>
       </c>
@@ -17595,7 +17595,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="297" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>144</v>
       </c>
@@ -17651,7 +17651,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="298" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>145</v>
       </c>
@@ -17707,7 +17707,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="299" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>145</v>
       </c>
@@ -17763,7 +17763,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="300" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>146</v>
       </c>
@@ -17819,7 +17819,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="301" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>146</v>
       </c>
@@ -17875,7 +17875,7 @@
         <v>27120000</v>
       </c>
     </row>
-    <row r="302" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>129</v>
       </c>
@@ -17931,7 +17931,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="303" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>129</v>
       </c>
@@ -17987,7 +17987,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="304" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>135</v>
       </c>
@@ -18043,7 +18043,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="305" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>135</v>
       </c>
@@ -18099,7 +18099,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="306" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>136</v>
       </c>
@@ -18155,7 +18155,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="307" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>136</v>
       </c>
@@ -18211,7 +18211,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="308" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>137</v>
       </c>
@@ -18267,7 +18267,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="309" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>137</v>
       </c>
@@ -18323,7 +18323,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="310" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>137</v>
       </c>
@@ -18379,7 +18379,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="311" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>139</v>
       </c>
@@ -18435,7 +18435,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="312" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>139</v>
       </c>
@@ -18491,7 +18491,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="313" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>139</v>
       </c>
@@ -18547,7 +18547,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="314" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>140</v>
       </c>
@@ -18603,7 +18603,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="315" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>140</v>
       </c>
@@ -18659,7 +18659,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="316" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>140</v>
       </c>
@@ -18715,7 +18715,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="317" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>141</v>
       </c>
@@ -18771,7 +18771,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="318" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>141</v>
       </c>
@@ -18827,7 +18827,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="319" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>142</v>
       </c>
@@ -18883,7 +18883,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="320" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>142</v>
       </c>
@@ -18939,7 +18939,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="321" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>143</v>
       </c>
@@ -18995,7 +18995,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="322" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>143</v>
       </c>
@@ -19051,7 +19051,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="323" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>144</v>
       </c>
@@ -19107,7 +19107,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="324" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>144</v>
       </c>
@@ -19163,7 +19163,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="325" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>145</v>
       </c>
@@ -19219,7 +19219,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="326" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>145</v>
       </c>
@@ -19275,7 +19275,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="327" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>146</v>
       </c>
@@ -19331,7 +19331,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="328" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>146</v>
       </c>
@@ -19387,7 +19387,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="329" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>27</v>
       </c>
@@ -19413,7 +19413,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="330" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>27</v>
       </c>
@@ -19485,7 +19485,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="331" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>27</v>
       </c>
@@ -19557,7 +19557,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="332" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>27</v>
       </c>
@@ -19630,7 +19630,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="333" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>27</v>
       </c>
@@ -19702,7 +19702,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="334" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>27</v>
       </c>
@@ -19731,7 +19731,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="335" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>27</v>
       </c>
@@ -19803,7 +19803,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="336" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>27</v>
       </c>
@@ -19875,7 +19875,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="337" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>27</v>
       </c>
@@ -19948,7 +19948,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="338" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>27</v>
       </c>
@@ -20020,7 +20020,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="339" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>27</v>
       </c>
@@ -20046,7 +20046,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="340" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>27</v>
       </c>
@@ -20118,7 +20118,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="341" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>27</v>
       </c>
@@ -20190,7 +20190,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="342" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>27</v>
       </c>
@@ -20263,7 +20263,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="343" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>27</v>
       </c>
@@ -20335,7 +20335,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="344" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>29</v>
       </c>
@@ -20361,7 +20361,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="345" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>29</v>
       </c>
@@ -20430,7 +20430,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="346" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>29</v>
       </c>
@@ -20499,7 +20499,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="347" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>29</v>
       </c>
@@ -20572,7 +20572,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="348" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>29</v>
       </c>
@@ -20641,7 +20641,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="349" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>29</v>
       </c>
@@ -20667,7 +20667,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="350" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>29</v>
       </c>
@@ -20736,7 +20736,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="351" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>29</v>
       </c>
@@ -20805,7 +20805,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="352" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>29</v>
       </c>
@@ -20878,7 +20878,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="353" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>29</v>
       </c>
@@ -20947,7 +20947,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="354" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>21</v>
       </c>
@@ -20976,7 +20976,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="355" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>21</v>
       </c>
@@ -21048,7 +21048,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="356" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>21</v>
       </c>
@@ -21120,7 +21120,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="357" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>21</v>
       </c>
@@ -21193,7 +21193,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="358" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>21</v>
       </c>
@@ -21265,7 +21265,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="359" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>21</v>
       </c>
@@ -21291,7 +21291,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="360" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>21</v>
       </c>
@@ -21363,7 +21363,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="361" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>21</v>
       </c>
@@ -21435,7 +21435,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="362" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>21</v>
       </c>
@@ -21508,7 +21508,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="363" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>21</v>
       </c>
@@ -21580,7 +21580,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="364" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>21</v>
       </c>
@@ -21606,7 +21606,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="365" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>21</v>
       </c>
@@ -21678,7 +21678,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="366" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>21</v>
       </c>
@@ -21750,7 +21750,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="367" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>21</v>
       </c>
@@ -21823,7 +21823,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="368" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>21</v>
       </c>
@@ -21895,7 +21895,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="369" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
         <v>21</v>
       </c>
@@ -21921,7 +21921,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="370" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>21</v>
       </c>
@@ -21993,7 +21993,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="371" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>21</v>
       </c>
@@ -22065,7 +22065,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="372" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>21</v>
       </c>
@@ -22138,7 +22138,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="373" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>21</v>
       </c>
@@ -22210,7 +22210,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="374" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>165</v>
       </c>
@@ -22236,7 +22236,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="375" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>165</v>
       </c>
@@ -22305,7 +22305,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="376" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>165</v>
       </c>
@@ -22377,7 +22377,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="377" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>165</v>
       </c>
@@ -22450,7 +22450,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="378" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>165</v>
       </c>
@@ -22522,7 +22522,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="379" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>165</v>
       </c>
@@ -22548,7 +22548,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="380" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>165</v>
       </c>
@@ -22617,7 +22617,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="381" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>165</v>
       </c>
@@ -22689,7 +22689,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="382" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>165</v>
       </c>
@@ -22762,7 +22762,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="383" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>165</v>
       </c>
@@ -22834,7 +22834,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="384" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>165</v>
       </c>
@@ -22860,7 +22860,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="385" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>165</v>
       </c>
@@ -22929,7 +22929,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="386" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>165</v>
       </c>
@@ -23001,7 +23001,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="387" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>165</v>
       </c>
@@ -23074,7 +23074,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="388" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>165</v>
       </c>
@@ -23146,7 +23146,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="389" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>165</v>
       </c>
@@ -23172,7 +23172,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="390" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>165</v>
       </c>
@@ -23241,7 +23241,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="391" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
         <v>165</v>
       </c>
@@ -23313,7 +23313,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="392" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
         <v>165</v>
       </c>
@@ -23386,7 +23386,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="393" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
         <v>165</v>
       </c>
@@ -23458,7 +23458,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="394" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
         <v>165</v>
       </c>
@@ -23484,7 +23484,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="395" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A395" t="s">
         <v>165</v>
       </c>
@@ -23553,7 +23553,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="396" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
         <v>165</v>
       </c>
@@ -23625,7 +23625,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="397" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
         <v>165</v>
       </c>
@@ -23698,7 +23698,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="398" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
         <v>165</v>
       </c>
@@ -23770,7 +23770,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="399" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
         <v>31</v>
       </c>
@@ -23796,7 +23796,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="400" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
         <v>31</v>
       </c>
@@ -23865,7 +23865,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="401" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
         <v>31</v>
       </c>
@@ -23934,7 +23934,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="402" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
         <v>31</v>
       </c>
@@ -24007,7 +24007,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="403" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
         <v>31</v>
       </c>
@@ -24076,7 +24076,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="404" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
         <v>31</v>
       </c>
@@ -24102,7 +24102,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="405" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
         <v>31</v>
       </c>
@@ -24171,7 +24171,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="406" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
         <v>31</v>
       </c>
@@ -24240,7 +24240,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="407" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
         <v>31</v>
       </c>
@@ -24313,7 +24313,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="408" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A408" t="s">
         <v>31</v>
       </c>
@@ -24382,7 +24382,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="409" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A409" t="s">
         <v>31</v>
       </c>
@@ -24408,7 +24408,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="410" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A410" t="s">
         <v>31</v>
       </c>
@@ -24477,7 +24477,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="411" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A411" t="s">
         <v>31</v>
       </c>
@@ -24546,7 +24546,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="412" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A412" t="s">
         <v>31</v>
       </c>
@@ -24619,7 +24619,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="413" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A413" t="s">
         <v>31</v>
       </c>
@@ -24688,7 +24688,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="414" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A414" t="s">
         <v>31</v>
       </c>
@@ -24714,7 +24714,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="415" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A415" t="s">
         <v>31</v>
       </c>
@@ -24783,7 +24783,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="416" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A416" t="s">
         <v>31</v>
       </c>
@@ -24852,7 +24852,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="417" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
         <v>31</v>
       </c>
@@ -24925,7 +24925,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="418" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
         <v>31</v>
       </c>
@@ -24994,7 +24994,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="419" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
         <v>31</v>
       </c>
@@ -25020,7 +25020,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="420" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A420" t="s">
         <v>31</v>
       </c>
@@ -25089,7 +25089,7 @@
         <v>0.39</v>
       </c>
     </row>
-    <row r="421" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
         <v>31</v>
       </c>
@@ -25158,7 +25158,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="422" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
         <v>31</v>
       </c>
@@ -25231,7 +25231,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="423" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
         <v>31</v>
       </c>
@@ -25300,7 +25300,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="424" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
         <v>31</v>
       </c>
@@ -25326,7 +25326,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="425" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A425" t="s">
         <v>31</v>
       </c>
@@ -25395,7 +25395,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="426" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A426" t="s">
         <v>31</v>
       </c>
@@ -25464,7 +25464,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="427" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
         <v>31</v>
       </c>
@@ -25537,7 +25537,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="428" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
         <v>31</v>
       </c>
@@ -25606,7 +25606,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="429" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
         <v>35</v>
       </c>
@@ -25632,7 +25632,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="430" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
         <v>35</v>
       </c>
@@ -25701,7 +25701,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="431" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A431" t="s">
         <v>35</v>
       </c>
@@ -25770,7 +25770,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="432" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
         <v>35</v>
       </c>
@@ -25843,7 +25843,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="433" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A433" t="s">
         <v>35</v>
       </c>
@@ -25912,7 +25912,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="434" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A434" t="s">
         <v>35</v>
       </c>
@@ -25938,7 +25938,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="435" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A435" t="s">
         <v>35</v>
       </c>
@@ -26007,7 +26007,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="436" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A436" t="s">
         <v>35</v>
       </c>
@@ -26076,7 +26076,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="437" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A437" t="s">
         <v>35</v>
       </c>
@@ -26149,7 +26149,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="438" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A438" t="s">
         <v>35</v>
       </c>
@@ -26218,7 +26218,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="439" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A439" t="s">
         <v>35</v>
       </c>
@@ -26244,7 +26244,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="440" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A440" t="s">
         <v>35</v>
       </c>
@@ -26313,7 +26313,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="441" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A441" t="s">
         <v>35</v>
       </c>
@@ -26382,7 +26382,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="442" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A442" t="s">
         <v>35</v>
       </c>
@@ -26455,7 +26455,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="443" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A443" t="s">
         <v>35</v>
       </c>
@@ -26524,7 +26524,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="444" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A444" t="s">
         <v>35</v>
       </c>
@@ -26550,7 +26550,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="445" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A445" t="s">
         <v>35</v>
       </c>
@@ -26619,7 +26619,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="446" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A446" t="s">
         <v>35</v>
       </c>
@@ -26688,7 +26688,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="447" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A447" t="s">
         <v>35</v>
       </c>
@@ -26761,7 +26761,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="448" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
         <v>35</v>
       </c>
@@ -26830,7 +26830,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="449" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
         <v>35</v>
       </c>
@@ -26856,7 +26856,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="450" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A450" t="s">
         <v>35</v>
       </c>
@@ -26925,7 +26925,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="451" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A451" t="s">
         <v>35</v>
       </c>
@@ -26994,7 +26994,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="452" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A452" t="s">
         <v>35</v>
       </c>
@@ -27067,7 +27067,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="453" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A453" t="s">
         <v>35</v>
       </c>
@@ -27136,7 +27136,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="454" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A454" t="s">
         <v>35</v>
       </c>
@@ -27162,7 +27162,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="455" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A455" t="s">
         <v>35</v>
       </c>
@@ -27231,7 +27231,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="456" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A456" t="s">
         <v>35</v>
       </c>
@@ -27300,7 +27300,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="457" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A457" t="s">
         <v>35</v>
       </c>
@@ -27373,7 +27373,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="458" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A458" t="s">
         <v>35</v>
       </c>
@@ -27442,7 +27442,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="459" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A459" t="s">
         <v>37</v>
       </c>
@@ -27468,7 +27468,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="460" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A460" t="s">
         <v>37</v>
       </c>
@@ -27537,7 +27537,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="461" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A461" t="s">
         <v>37</v>
       </c>
@@ -27606,7 +27606,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="462" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A462" t="s">
         <v>37</v>
       </c>
@@ -27679,7 +27679,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="463" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A463" t="s">
         <v>37</v>
       </c>
@@ -27748,7 +27748,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="464" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A464" t="s">
         <v>37</v>
       </c>
@@ -27774,7 +27774,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="465" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A465" t="s">
         <v>37</v>
       </c>
@@ -27843,7 +27843,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="466" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A466" t="s">
         <v>37</v>
       </c>
@@ -27912,7 +27912,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="467" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A467" t="s">
         <v>37</v>
       </c>
@@ -27985,7 +27985,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="468" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A468" t="s">
         <v>37</v>
       </c>
@@ -28054,7 +28054,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="469" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A469" t="s">
         <v>37</v>
       </c>
@@ -28080,7 +28080,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="470" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A470" t="s">
         <v>37</v>
       </c>
@@ -28149,7 +28149,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="471" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A471" t="s">
         <v>37</v>
       </c>
@@ -28218,7 +28218,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="472" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A472" t="s">
         <v>37</v>
       </c>
@@ -28291,7 +28291,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="473" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A473" t="s">
         <v>37</v>
       </c>
@@ -28360,7 +28360,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="474" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A474" t="s">
         <v>40</v>
       </c>
@@ -28386,7 +28386,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="475" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A475" t="s">
         <v>40</v>
       </c>
@@ -28455,7 +28455,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="476" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A476" t="s">
         <v>40</v>
       </c>
@@ -28524,7 +28524,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="477" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A477" t="s">
         <v>40</v>
       </c>
@@ -28597,7 +28597,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="478" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A478" t="s">
         <v>40</v>
       </c>
@@ -28666,7 +28666,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="479" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A479" t="s">
         <v>40</v>
       </c>
@@ -28692,7 +28692,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="480" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A480" t="s">
         <v>40</v>
       </c>
@@ -28761,7 +28761,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="481" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A481" t="s">
         <v>40</v>
       </c>
@@ -28830,7 +28830,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="482" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A482" t="s">
         <v>40</v>
       </c>
@@ -28903,7 +28903,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="483" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A483" t="s">
         <v>40</v>
       </c>
@@ -28972,7 +28972,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="484" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A484" t="s">
         <v>189</v>
       </c>
@@ -28998,7 +28998,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="485" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A485" t="s">
         <v>189</v>
       </c>
@@ -29067,7 +29067,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="486" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A486" t="s">
         <v>189</v>
       </c>
@@ -29136,7 +29136,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="487" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A487" t="s">
         <v>189</v>
       </c>
@@ -29205,7 +29205,7 @@
         <v>92227251.175370395</v>
       </c>
     </row>
-    <row r="488" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A488" t="s">
         <v>189</v>
       </c>

</xml_diff>